<commit_message>
added to git ignore
</commit_message>
<xml_diff>
--- a/inData_Michal/Patogeny_hmyz_postbrouk_1.xlsx
+++ b/inData_Michal/Patogeny_hmyz_postbrouk_1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{F8E77651-1DC1-42E0-AAC2-83D9073A7399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{710B72A8-1131-4B7F-AC3C-94BE42B4C0A8}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3D3423D8-813C-44BA-B149-D0D6E988FD1F}"/>
+    <workbookView xWindow="1480" yWindow="1480" windowWidth="28800" windowHeight="15370" xr2:uid="{3D3423D8-813C-44BA-B149-D0D6E988FD1F}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -3650,6 +3650,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Neugebauer Michal" refreshedDate="46190.636003587962" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="122" xr:uid="{5AB3941F-5DC2-483C-B949-E924D041DCE0}">
   <cacheSource type="worksheet">
@@ -5092,16 +5096,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D134315-1AC4-413A-9A9F-A8F0E558586D}">
   <dimension ref="A1:E122"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" style="11" customWidth="1"/>
-    <col min="5" max="5" width="46.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="4" max="4" width="26.90625" style="11" customWidth="1"/>
+    <col min="5" max="5" width="46.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>124</v>
       </c>
@@ -5118,7 +5122,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C2" s="5" t="s">
         <v>95</v>
       </c>
@@ -5129,7 +5133,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C3" s="5" t="s">
         <v>86</v>
       </c>
@@ -5140,7 +5144,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C4" s="5" t="s">
         <v>89</v>
       </c>
@@ -5151,7 +5155,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C5" s="3" t="s">
         <v>27</v>
       </c>
@@ -5162,7 +5166,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C6" s="3" t="s">
         <v>57</v>
       </c>
@@ -5173,7 +5177,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C7" s="3" t="s">
         <v>71</v>
       </c>
@@ -5184,7 +5188,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C8" s="3" t="s">
         <v>74</v>
       </c>
@@ -5195,7 +5199,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C9" s="3" t="s">
         <v>97</v>
       </c>
@@ -5206,7 +5210,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C10" s="3" t="s">
         <v>7</v>
       </c>
@@ -5217,7 +5221,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C11" s="3" t="s">
         <v>30</v>
       </c>
@@ -5228,7 +5232,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C12" s="3" t="s">
         <v>32</v>
       </c>
@@ -5239,7 +5243,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C13" s="3" t="s">
         <v>36</v>
       </c>
@@ -5250,7 +5254,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C14" s="3" t="s">
         <v>20</v>
       </c>
@@ -5261,7 +5265,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C15" s="3" t="s">
         <v>38</v>
       </c>
@@ -5272,7 +5276,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C16" s="3" t="s">
         <v>21</v>
       </c>
@@ -5283,7 +5287,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C17" s="3" t="s">
         <v>39</v>
       </c>
@@ -5294,7 +5298,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C18" s="3" t="s">
         <v>22</v>
       </c>
@@ -5305,7 +5309,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C19" s="3" t="s">
         <v>40</v>
       </c>
@@ -5316,7 +5320,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C20" s="3" t="s">
         <v>41</v>
       </c>
@@ -5327,7 +5331,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C21" s="3" t="s">
         <v>42</v>
       </c>
@@ -5338,7 +5342,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C22" s="3" t="s">
         <v>23</v>
       </c>
@@ -5349,7 +5353,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="23" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C23" s="3" t="s">
         <v>24</v>
       </c>
@@ -5360,7 +5364,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C24" s="3" t="s">
         <v>43</v>
       </c>
@@ -5371,7 +5375,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="25" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C25" s="3" t="s">
         <v>44</v>
       </c>
@@ -5382,7 +5386,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="26" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C26" s="3" t="s">
         <v>45</v>
       </c>
@@ -5393,7 +5397,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C27" s="3" t="s">
         <v>46</v>
       </c>
@@ -5404,7 +5408,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="28" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C28" s="3" t="s">
         <v>47</v>
       </c>
@@ -5415,7 +5419,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="29" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C29" s="3" t="s">
         <v>51</v>
       </c>
@@ -5426,7 +5430,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="30" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C30" s="3" t="s">
         <v>52</v>
       </c>
@@ -5437,7 +5441,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="31" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C31" s="3" t="s">
         <v>53</v>
       </c>
@@ -5448,7 +5452,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="32" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C32" s="3" t="s">
         <v>54</v>
       </c>
@@ -5459,7 +5463,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="33" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C33" s="3" t="s">
         <v>55</v>
       </c>
@@ -5470,7 +5474,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="34" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C34" s="3" t="s">
         <v>61</v>
       </c>
@@ -5481,7 +5485,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="35" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C35" s="3" t="s">
         <v>64</v>
       </c>
@@ -5492,7 +5496,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="36" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C36" s="3" t="s">
         <v>65</v>
       </c>
@@ -5503,7 +5507,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="37" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C37" s="3" t="s">
         <v>66</v>
       </c>
@@ -5514,7 +5518,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="38" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C38" s="3" t="s">
         <v>70</v>
       </c>
@@ -5525,7 +5529,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="39" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C39" s="3" t="s">
         <v>78</v>
       </c>
@@ -5536,7 +5540,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="40" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C40" s="3" t="s">
         <v>25</v>
       </c>
@@ -5547,7 +5551,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="41" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C41" s="3" t="s">
         <v>93</v>
       </c>
@@ -5558,7 +5562,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="42" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C42" s="3" t="s">
         <v>28</v>
       </c>
@@ -5569,7 +5573,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="43" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C43" s="3" t="s">
         <v>33</v>
       </c>
@@ -5580,7 +5584,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="44" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C44" s="3" t="s">
         <v>15</v>
       </c>
@@ -5591,7 +5595,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="45" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C45" s="3" t="s">
         <v>37</v>
       </c>
@@ -5602,7 +5606,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="46" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C46" s="3" t="s">
         <v>19</v>
       </c>
@@ -5613,7 +5617,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="47" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C47" s="3" t="s">
         <v>48</v>
       </c>
@@ -5624,7 +5628,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="48" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C48" s="3" t="s">
         <v>49</v>
       </c>
@@ -5635,7 +5639,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="49" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C49" s="3" t="s">
         <v>57</v>
       </c>
@@ -5646,7 +5650,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="50" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C50" s="3" t="s">
         <v>63</v>
       </c>
@@ -5657,7 +5661,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="51" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C51" s="3" t="s">
         <v>69</v>
       </c>
@@ -5668,7 +5672,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="52" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C52" s="3" t="s">
         <v>33</v>
       </c>
@@ -5679,7 +5683,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C53" s="3" t="s">
         <v>3</v>
       </c>
@@ -5690,7 +5694,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="54" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C54" s="3" t="s">
         <v>6</v>
       </c>
@@ -5701,7 +5705,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="55" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C55" s="3" t="s">
         <v>10</v>
       </c>
@@ -5712,7 +5716,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="56" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C56" s="3" t="s">
         <v>11</v>
       </c>
@@ -5723,7 +5727,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="57" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C57" s="3" t="s">
         <v>12</v>
       </c>
@@ -5734,7 +5738,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C58" s="3" t="s">
         <v>18</v>
       </c>
@@ -5745,7 +5749,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="59" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C59" s="3" t="s">
         <v>1</v>
       </c>
@@ -5756,7 +5760,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="60" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C60" s="3" t="s">
         <v>26</v>
       </c>
@@ -5767,7 +5771,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="61" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C61" s="3" t="s">
         <v>50</v>
       </c>
@@ -5778,7 +5782,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="62" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C62" s="3" t="s">
         <v>75</v>
       </c>
@@ -5789,7 +5793,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="63" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C63" s="3" t="s">
         <v>76</v>
       </c>
@@ -5800,7 +5804,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="64" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C64" s="3" t="s">
         <v>77</v>
       </c>
@@ -5811,7 +5815,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="65" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C65" s="3" t="s">
         <v>83</v>
       </c>
@@ -5822,7 +5826,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="66" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C66" s="3" t="s">
         <v>16</v>
       </c>
@@ -5833,7 +5837,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="67" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C67" s="3" t="s">
         <v>4</v>
       </c>
@@ -5844,7 +5848,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="68" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C68" s="3" t="s">
         <v>72</v>
       </c>
@@ -5855,7 +5859,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="69" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C69" s="3" t="s">
         <v>67</v>
       </c>
@@ -5866,7 +5870,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="70" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C70" s="3" t="s">
         <v>35</v>
       </c>
@@ -5877,7 +5881,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="71" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C71" s="3" t="s">
         <v>62</v>
       </c>
@@ -5888,7 +5892,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="72" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C72" s="3" t="s">
         <v>58</v>
       </c>
@@ -5899,7 +5903,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="73" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C73" s="3" t="s">
         <v>29</v>
       </c>
@@ -5910,7 +5914,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="74" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C74" s="3" t="s">
         <v>56</v>
       </c>
@@ -5921,7 +5925,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="75" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C75" s="3" t="s">
         <v>31</v>
       </c>
@@ -5932,7 +5936,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="76" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C76" s="3" t="s">
         <v>34</v>
       </c>
@@ -5943,7 +5947,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="77" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C77" s="3" t="s">
         <v>79</v>
       </c>
@@ -5954,7 +5958,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="78" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C78" s="3" t="s">
         <v>80</v>
       </c>
@@ -5965,7 +5969,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="79" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C79" s="3" t="s">
         <v>81</v>
       </c>
@@ -5976,7 +5980,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="80" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C80" s="3" t="s">
         <v>82</v>
       </c>
@@ -5987,7 +5991,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C81" s="3" t="s">
         <v>88</v>
       </c>
@@ -5998,7 +6002,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C82" s="3" t="s">
         <v>92</v>
       </c>
@@ -6009,7 +6013,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C83" s="5" t="s">
         <v>93</v>
       </c>
@@ -6020,7 +6024,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C84" s="3" t="s">
         <v>49</v>
       </c>
@@ -6031,7 +6035,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C85" s="3" t="s">
         <v>59</v>
       </c>
@@ -6042,7 +6046,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>145</v>
       </c>
@@ -6059,7 +6063,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>145</v>
       </c>
@@ -6076,7 +6080,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>146</v>
       </c>
@@ -6093,7 +6097,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>146</v>
       </c>
@@ -6110,7 +6114,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>147</v>
       </c>
@@ -6127,7 +6131,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>147</v>
       </c>
@@ -6144,7 +6148,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>148</v>
       </c>
@@ -6161,7 +6165,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>149</v>
       </c>
@@ -6178,7 +6182,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>149</v>
       </c>
@@ -6195,7 +6199,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>150</v>
       </c>
@@ -6212,7 +6216,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>150</v>
       </c>
@@ -6229,7 +6233,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>151</v>
       </c>
@@ -6246,7 +6250,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>125</v>
       </c>
@@ -6263,7 +6267,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>125</v>
       </c>
@@ -6280,7 +6284,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>126</v>
       </c>
@@ -6297,7 +6301,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>127</v>
       </c>
@@ -6314,7 +6318,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>128</v>
       </c>
@@ -6331,7 +6335,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>129</v>
       </c>
@@ -6348,7 +6352,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>130</v>
       </c>
@@ -6365,7 +6369,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>130</v>
       </c>
@@ -6382,7 +6386,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>131</v>
       </c>
@@ -6399,7 +6403,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>132</v>
       </c>
@@ -6416,7 +6420,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>133</v>
       </c>
@@ -6433,7 +6437,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>134</v>
       </c>
@@ -6450,7 +6454,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>135</v>
       </c>
@@ -6467,7 +6471,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>136</v>
       </c>
@@ -6484,7 +6488,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>137</v>
       </c>
@@ -6501,7 +6505,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>137</v>
       </c>
@@ -6518,7 +6522,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>138</v>
       </c>
@@ -6535,7 +6539,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>139</v>
       </c>
@@ -6552,7 +6556,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>139</v>
       </c>
@@ -6569,7 +6573,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>140</v>
       </c>
@@ -6586,7 +6590,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>141</v>
       </c>
@@ -6603,7 +6607,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>142</v>
       </c>
@@ -6620,7 +6624,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>142</v>
       </c>
@@ -6637,7 +6641,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>143</v>
       </c>
@@ -6654,7 +6658,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>144</v>
       </c>
@@ -6680,14 +6684,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E970006-4B8D-4DA4-B79E-C1B6F4633952}">
   <dimension ref="B3:D28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="26.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="6" t="s">
         <v>108</v>
       </c>
@@ -6698,7 +6702,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B4" s="7" t="s">
         <v>84</v>
       </c>
@@ -6709,7 +6713,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B5" s="7" t="s">
         <v>8</v>
       </c>
@@ -6720,7 +6724,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="7" t="s">
         <v>2</v>
       </c>
@@ -6731,7 +6735,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="7" t="s">
         <v>5</v>
       </c>
@@ -6742,7 +6746,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="7" t="s">
         <v>13</v>
       </c>
@@ -6753,7 +6757,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="7" t="s">
         <v>0</v>
       </c>
@@ -6764,7 +6768,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B10" s="7" t="s">
         <v>91</v>
       </c>
@@ -6775,7 +6779,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B11" s="7" t="s">
         <v>102</v>
       </c>
@@ -6786,7 +6790,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B12" s="7" t="s">
         <v>14</v>
       </c>
@@ -6797,7 +6801,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="7" t="s">
         <v>98</v>
       </c>
@@ -6808,7 +6812,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B14" s="7" t="s">
         <v>87</v>
       </c>
@@ -6819,7 +6823,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B15" s="7" t="s">
         <v>99</v>
       </c>
@@ -6830,7 +6834,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B16" s="7" t="s">
         <v>94</v>
       </c>
@@ -6838,7 +6842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B17" s="7" t="s">
         <v>96</v>
       </c>
@@ -6849,7 +6853,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B18" s="7" t="s">
         <v>103</v>
       </c>
@@ -6860,7 +6864,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B19" s="7" t="s">
         <v>101</v>
       </c>
@@ -6871,7 +6875,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B20" s="7" t="s">
         <v>85</v>
       </c>
@@ -6882,7 +6886,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B21" s="7" t="s">
         <v>9</v>
       </c>
@@ -6893,7 +6897,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B22" s="7" t="s">
         <v>73</v>
       </c>
@@ -6904,7 +6908,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B23" s="7" t="s">
         <v>68</v>
       </c>
@@ -6915,7 +6919,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B24" s="7" t="s">
         <v>90</v>
       </c>
@@ -6923,7 +6927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B25" s="7" t="s">
         <v>60</v>
       </c>
@@ -6934,7 +6938,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B26" s="7" t="s">
         <v>17</v>
       </c>
@@ -6945,7 +6949,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B27" s="7" t="s">
         <v>100</v>
       </c>
@@ -6956,7 +6960,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B28" s="7" t="s">
         <v>104</v>
       </c>
@@ -6983,6 +6987,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100082E014C7AAC9D4D9EA25F6BE03BD2B0" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc843cee3e1e3e71d005a4bfa49a4ddc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e3a1a65f-a950-4f4e-91c6-450504a86f87" xmlns:ns3="514d2724-d259-4a80-ac9f-15d3c2594ecd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="58a2d892520dfae734554831702004e8" ns2:_="" ns3:_="">
     <xsd:import namespace="e3a1a65f-a950-4f4e-91c6-450504a86f87"/>
@@ -7217,15 +7230,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{653A886F-B326-4709-9ED0-D3DE8D23A1CA}">
   <ds:schemaRefs>
@@ -7238,6 +7242,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A90DEA9-1655-407E-9BCF-8D5F791F2979}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE583EB-B534-4EC1-B56B-C41957A3B188}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7256,10 +7268,8 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A90DEA9-1655-407E-9BCF-8D5F791F2979}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f26a48e1-fc21-461a-b97f-ac5bd535f341}" enabled="0" method="" siteId="{f26a48e1-fc21-461a-b97f-ac5bd535f341}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>